<commit_message>
Backfill reports (HTML + XLSX)
</commit_message>
<xml_diff>
--- a/reports/2025-12-01/category_report.xlsx
+++ b/reports/2025-12-01/category_report.xlsx
@@ -413,11 +413,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -453,20 +453,286 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>B- TASTING</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>459</v>
+      </c>
+      <c r="C2" t="n">
+        <v>459</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BEER</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2943.64</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3385.24</v>
+      </c>
+      <c r="D3" t="n">
+        <v>286</v>
+      </c>
+      <c r="E3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>COOLCIDER</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1668.47</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1918.85</v>
+      </c>
+      <c r="D4" t="n">
+        <v>167</v>
+      </c>
+      <c r="E4" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Deposit</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>229.6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>229.6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>756</v>
+      </c>
+      <c r="E5" t="n">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>L-TASTING</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>851</v>
+      </c>
+      <c r="C6" t="n">
+        <v>851</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>R -TASTING</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>225</v>
+      </c>
+      <c r="C7" t="n">
+        <v>225</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RETAIL</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>55.37</v>
+      </c>
+      <c r="C8" t="n">
+        <v>58.43</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Returns</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-28</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rewards</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>-120</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-120</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-24</v>
+      </c>
+      <c r="E10" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SPIRITS</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3267.45</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3757.61</v>
+      </c>
+      <c r="D11" t="n">
+        <v>137</v>
+      </c>
+      <c r="E11" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>W-TASTING</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>206</v>
+      </c>
+      <c r="C12" t="n">
+        <v>206</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WINE</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>693.79</v>
+      </c>
+      <c r="C13" t="n">
+        <v>797.87</v>
+      </c>
+      <c r="D13" t="n">
+        <v>25</v>
+      </c>
+      <c r="E13" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WINE RED</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1379.58</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1586.59</v>
+      </c>
+      <c r="D14" t="n">
+        <v>74</v>
+      </c>
+      <c r="E14" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WINE WHITE</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1124.22</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1292.88</v>
+      </c>
+      <c r="D15" t="n">
+        <v>61</v>
+      </c>
+      <c r="E15" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
+      <c r="B16" t="n">
+        <v>12980.32</v>
+      </c>
+      <c r="C16" t="n">
+        <v>14645.27</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1473</v>
+      </c>
+      <c r="E16" t="n">
+        <v>361</v>
       </c>
     </row>
   </sheetData>

</xml_diff>